<commit_message>
pre-refactor: _guardar_acumuladas formato simple antes de migrar a exportar_trazabilidad
</commit_message>
<xml_diff>
--- a/shared/usuarios_id.xlsx
+++ b/shared/usuarios_id.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilde\PycharmProjects\jass_system\03_pagos\yape\construir_maestro\Inputs\Usuario id\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilde\PycharmProjects\jass_system\shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3CBD210-423D-4B15-A88D-3B45D4C13867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B6AF45C-AC1C-42F1-A0A5-EF97E5B1A710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28230" yWindow="570" windowWidth="14610" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="usuarios_id" sheetId="1" r:id="rId1"/>
@@ -3711,7 +3711,7 @@
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="6" customWidth="1"/>
+    <col min="5" max="5" width="6.6328125" customWidth="1"/>
     <col min="6" max="6" width="7" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
fix(4_pagos/efectivo): corrige lotes mal escritos en mesa_1/mesa_2 verificados a mano
Fotos nuevas de la secretaria contra usuarios_id.xlsx destaparon 2 errores reales
(M-19->M-14 "Magda", G-13->O-13 "Pedro") y confirmaron W-2->U-2 en la mesa de
Wilder. Se agrega un BLANCO de S/16 del 01/08 (mismo patrón que el de S/49 del
02/08 ya existente).

shared/usuarios_id.xlsx: crea U0500 (M-12, Ramon Requez Mendoza, existia en
0_padron/planilla pero nunca se cargo aca) y corrige U0457 de C1-17 a C1-9
(el override de julio nunca lo actualizo).

entregas_hoja.xlsx: declara Wilder 01/08 (595, del "recibi" tachado en el papel)
y Yerald 01/08+02/08 (asumidos = lo que registra mesa_2.xlsx, sus fotos no
traen una declaracion "Recibi X" legible como Wilder) con nota aclaratoria.
</commit_message>
<xml_diff>
--- a/shared/usuarios_id.xlsx
+++ b/shared/usuarios_id.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F497"/>
+  <dimension ref="A1:F498"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11453,7 +11453,7 @@
       </c>
       <c r="D455" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E455" s="4" t="n"/>
@@ -12466,6 +12466,30 @@
       </c>
       <c r="E497" s="4" t="n"/>
       <c r="F497" s="4" t="n"/>
+    </row>
+    <row r="498">
+      <c r="A498" s="4" t="inlineStr">
+        <is>
+          <t>U0500</t>
+        </is>
+      </c>
+      <c r="B498" s="5" t="inlineStr">
+        <is>
+          <t>RAMON REQUEZ MENDOZA</t>
+        </is>
+      </c>
+      <c r="C498" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D498" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E498" s="4" t="n"/>
+      <c r="F498" s="4" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F497"/>

</xml_diff>